<commit_message>
[UPDATE] Updated test files P.DINAMICO and P.INMOBILIARIO
</commit_message>
<xml_diff>
--- a/test_files/BTG_P.DINAMICO_EEFF_2025-06-30.xlsx
+++ b/test_files/BTG_P.DINAMICO_EEFF_2025-06-30.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDriveUniversidad EIA\Documentos\Valen\BTG Pactual\Proyectos\iastronauts_creditiq\test_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E077FE6F-9653-43A3-A64C-18C4335A5CA9}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31261DBC-7DC9-4274-BEDE-B6803C59AC58}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BALANCE" sheetId="1" r:id="rId1"/>
@@ -32,12 +32,19 @@
     <sheet name="GASTOS_ADM" sheetId="17" r:id="rId17"/>
     <sheet name="RIESGOS" sheetId="18" r:id="rId18"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="179021"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="163">
   <si>
     <t>JUNIO 2025</t>
   </si>
@@ -360,24 +367,6 @@
     <t>28,657</t>
   </si>
   <si>
-    <t>Cementos Argos</t>
-  </si>
-  <si>
-    <t>BAC Holding</t>
-  </si>
-  <si>
-    <t>BTG Fondo Liquidez</t>
-  </si>
-  <si>
-    <t>Almacenes Éxito</t>
-  </si>
-  <si>
-    <t>Bancolombia</t>
-  </si>
-  <si>
-    <t>Subtotal Instrumentos de Patrimonio</t>
-  </si>
-  <si>
     <t>Gobierno de la Unión Europea</t>
   </si>
   <si>
@@ -508,16 +497,53 @@
   </si>
   <si>
     <t>VL 2024</t>
+  </si>
+  <si>
+    <t>Subtotal</t>
+  </si>
+  <si>
+    <t>Btg Pactual Fondo Liquidez</t>
+  </si>
+  <si>
+    <t>Invesco QQQ Trust Series 1</t>
+  </si>
+  <si>
+    <t>Ishares Core s&amp;p 500 UCITS</t>
+  </si>
+  <si>
+    <t>Interconexión eléctrica S.A E.S.P</t>
+  </si>
+  <si>
+    <t>Suzano sa</t>
+  </si>
+  <si>
+    <t>Teleperformance</t>
+  </si>
+  <si>
+    <t>Apple INC</t>
+  </si>
+  <si>
+    <t>Btg Pactual Fondo Acciones Colombia</t>
+  </si>
+  <si>
+    <t>Btg Pactual Fondo Deuda Privada</t>
+  </si>
+  <si>
+    <t>Ishares Corp Bond UCITS ETF</t>
+  </si>
+  <si>
+    <t>Vanguard USD Treasury Bond UCITS ETF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="\$\ #,##0;[Red]\-\$\ #,##0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -554,6 +580,18 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -642,10 +680,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -669,6 +708,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -688,8 +728,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1146,12 +1193,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1242,7 +1289,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="7" customWidth="1"/>
@@ -1253,22 +1300,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1319,204 +1366,290 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3">
+        <f>+SUM(C4:C5)</f>
+        <v>17680566</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3">
+        <f>+SUM(E4:E5)</f>
+        <v>12014360</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C7" s="3">
         <v>17680566</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E7" s="3">
         <v>12014360</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C7" s="3">
-        <v>2922898</v>
-      </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C8" s="3">
-        <v>1556566</v>
-      </c>
+    <row r="8" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
       <c r="D8" s="3"/>
-      <c r="E8" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>106</v>
-      </c>
+      <c r="E8" s="3"/>
+    </row>
+    <row r="9" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
+        <v>152</v>
+      </c>
+      <c r="B9" s="3"/>
       <c r="C9" s="3">
-        <v>1322807</v>
+        <v>3952756</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3">
-        <v>0</v>
+        <v>3270920</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B10" s="3">
-        <v>234673</v>
+        <v>101</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="C10" s="3">
-        <v>2417132</v>
-      </c>
-      <c r="D10" s="3">
-        <v>899276</v>
-      </c>
+        <v>2922898</v>
+      </c>
+      <c r="D10" s="3"/>
       <c r="E10" s="3">
-        <v>9172615</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B11" s="3">
-        <v>4960683</v>
+        <v>103</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="C11" s="3">
-        <v>1557654</v>
-      </c>
-      <c r="D11" s="3">
-        <v>8883827</v>
-      </c>
+        <v>1556566</v>
+      </c>
+      <c r="D11" s="3"/>
       <c r="E11" s="3">
-        <v>2647381</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" s="3">
-        <v>46959</v>
+        <v>105</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>106</v>
       </c>
       <c r="C12" s="3">
-        <v>970065</v>
-      </c>
-      <c r="D12" s="3">
-        <v>13818</v>
-      </c>
+        <v>1322807</v>
+      </c>
+      <c r="D12" s="3"/>
       <c r="E12" s="3">
-        <v>272412</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B13" s="3">
-        <v>224520</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="B13" s="3"/>
       <c r="C13" s="3">
-        <v>614062</v>
-      </c>
-      <c r="D13" s="3">
-        <v>0</v>
-      </c>
+        <v>773999</v>
+      </c>
+      <c r="D13" s="3"/>
       <c r="E13" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="B14" s="3">
-        <v>0</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="B14" s="3"/>
       <c r="C14" s="3">
-        <v>0</v>
-      </c>
-      <c r="D14" s="3">
-        <v>556071</v>
-      </c>
+        <v>624886</v>
+      </c>
+      <c r="D14" s="3"/>
       <c r="E14" s="3">
-        <v>19981862</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+        <v>2050469</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3">
+        <v>426041</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3">
+        <v>182730</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3">
+        <v>626042</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3">
+        <v>161423</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3">
+        <v>818</v>
+      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3">
+        <v>1112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3">
+        <v>4420999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3">
+        <v>480172</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3">
+        <v>2441139</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3">
+        <v>3465823</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3">
+        <v>4972223</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B24" s="4"/>
+      <c r="C24" s="5">
+        <f>+SUM(C9:C23)</f>
+        <v>11924924</v>
+      </c>
+      <c r="D24" s="4"/>
+      <c r="E24" s="5">
+        <f>+SUM(E9:E23)</f>
+        <v>21728899</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="29"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" s="29">
+        <v>4308</v>
+      </c>
+      <c r="E26" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="C27" s="29">
+        <v>4308</v>
+      </c>
+      <c r="E27" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="5">
-        <v>39521260</v>
-      </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="5">
-        <v>52559635</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="C18">
-        <v>11924924</v>
-      </c>
-      <c r="E18">
-        <v>21728899</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>113</v>
-      </c>
-      <c r="B20">
-        <v>4308</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="C21">
+      <c r="C28" s="29">
         <v>29609798</v>
       </c>
-      <c r="E21">
+      <c r="D28" s="29"/>
+      <c r="E28" s="29">
         <v>33743259</v>
       </c>
     </row>
@@ -1526,6 +1659,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1540,11 +1674,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
+      <c r="A1" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1559,7 +1693,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B4" s="3">
         <v>28347</v>
@@ -1570,7 +1704,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B5" s="3">
         <v>6157</v>
@@ -1581,7 +1715,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B6" s="3">
         <v>17</v>
@@ -1622,34 +1756,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="A1" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B4" s="3">
         <v>15.57</v>
@@ -1666,7 +1800,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B5" s="3">
         <v>15.22</v>
@@ -1683,7 +1817,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B6" s="3">
         <v>15.33</v>
@@ -1700,7 +1834,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B7" s="3">
         <v>14.99</v>
@@ -1717,7 +1851,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B8" s="3">
         <v>12.41</v>
@@ -1764,34 +1898,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>129</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="A1" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B4" s="3">
         <v>14.78</v>
@@ -1808,7 +1942,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B5" s="3">
         <v>14.58</v>
@@ -1825,7 +1959,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B6" s="3">
         <v>11.73</v>
@@ -1842,7 +1976,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B7" s="3">
         <v>14.49</v>
@@ -1859,7 +1993,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B8" s="3">
         <v>14.3</v>
@@ -1903,34 +2037,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="A1" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B4" s="3">
         <v>1692794</v>
@@ -1947,7 +2081,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B5" s="3">
         <v>489368</v>
@@ -1964,7 +2098,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B6" s="3">
         <v>264958</v>
@@ -1981,7 +2115,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="B7" s="3">
         <v>83167</v>
@@ -1998,7 +2132,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B8" s="3">
         <v>5143</v>
@@ -2015,7 +2149,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B9" s="3">
         <v>25</v>
@@ -2032,7 +2166,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="B10" s="3">
         <v>0</v>
@@ -2099,34 +2233,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>142</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="A1" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B4" s="3">
         <v>206530</v>
@@ -2143,7 +2277,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="B5" s="3">
         <v>119881</v>
@@ -2160,7 +2294,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="B6" s="5">
         <v>108295</v>
@@ -2177,7 +2311,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B7">
         <v>2882</v>
@@ -2227,34 +2361,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="A1" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B4" s="3">
         <v>224434</v>
@@ -2271,7 +2405,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="B5" s="3">
         <v>6550</v>
@@ -2288,7 +2422,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B6" s="3">
         <v>950</v>
@@ -2305,7 +2439,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B7" s="3">
         <v>675</v>
@@ -2322,7 +2456,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B8" s="3">
         <v>0</v>
@@ -2375,29 +2509,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>152</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="A1" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2505,14 +2639,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="16"/>
-      <c r="D1" s="15" t="s">
+      <c r="C1" s="17"/>
+      <c r="D1" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="16"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
@@ -2529,12 +2663,12 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="16"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="17"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -2686,10 +2820,10 @@
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="16"/>
+      <c r="C2" s="17"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -2775,10 +2909,10 @@
       <c r="A2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="16"/>
+      <c r="C2" s="17"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -2941,14 +3075,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="18" t="s">
+      <c r="C1" s="20"/>
+      <c r="D1" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="19"/>
+      <c r="E1" s="20"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" s="11" t="s">
@@ -3168,14 +3302,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="20" t="s">
+      <c r="C1" s="20"/>
+      <c r="D1" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="19"/>
+      <c r="E1" s="20"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
@@ -3264,14 +3398,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="18" t="s">
+      <c r="C1" s="20"/>
+      <c r="D1" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="19"/>
+      <c r="E1" s="20"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">

</xml_diff>